<commit_message>
feat: support self-hosted HTTP evidence sources
</commit_message>
<xml_diff>
--- a/input/05_input_bast.xlsx
+++ b/input/05_input_bast.xlsx
@@ -105,7 +105,7 @@
     <t>001</t>
   </si>
   <si>
-    <t>https://drive.google.com/open?id=1u87uDsnJTOAOBEGdiFob_NB_8ze9H8pw</t>
+    <t>https://example.go.id/api/dokumen/123/gambar</t>
   </si>
   <si>
     <t>TABUNGANEN</t>
@@ -123,7 +123,7 @@
     <t>002</t>
   </si>
   <si>
-    <t>https://drive.google.com/open?id=123QHoXuVKEk4zAKVS-fIBpYHAdkJX_ZW, https://drive.google.com/open?id=1ws8SS3egejgygItNiIAk1xxDxmCX--E1</t>
+    <t>https://example.go.id/api/dokumen/123/gambar, https://example.go.id/api/dokumen/123/gambar</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
feat: support universal evidence sources
Squashed changes from feat/self-hosted-evidence-source.
</commit_message>
<xml_diff>
--- a/input/05_input_bast.xlsx
+++ b/input/05_input_bast.xlsx
@@ -105,7 +105,7 @@
     <t>001</t>
   </si>
   <si>
-    <t>https://drive.google.com/open?id=1u87uDsnJTOAOBEGdiFob_NB_8ze9H8pw</t>
+    <t>https://example.go.id/api/dokumen/123/gambar</t>
   </si>
   <si>
     <t>TABUNGANEN</t>
@@ -123,7 +123,7 @@
     <t>002</t>
   </si>
   <si>
-    <t>https://drive.google.com/open?id=123QHoXuVKEk4zAKVS-fIBpYHAdkJX_ZW, https://drive.google.com/open?id=1ws8SS3egejgygItNiIAk1xxDxmCX--E1</t>
+    <t>https://example.go.id/api/dokumen/123/gambar, https://example.go.id/api/dokumen/123/gambar</t>
   </si>
 </sst>
 </file>

</xml_diff>